<commit_message>
Major changes: - Added a new data source abstraction layer to support both live and mock data sources.
</commit_message>
<xml_diff>
--- a/test data/2hire vehicle test data.xlsx
+++ b/test data/2hire vehicle test data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mh3dk-my.sharepoint.com/personal/jlk_mh3_dk/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mh3dk-my.sharepoint.com/personal/jlk_mh3_dk/Documents/Shared folders/Documents-FLEETii/FLEETii webapp/test data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{20DE8C20-266C-4DFF-8EE4-25CBA7ED4FE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47FE67E4-D81D-46D2-8C64-55F342214B6C}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{20DE8C20-266C-4DFF-8EE4-25CBA7ED4FE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B10F0250-8DDF-430F-8E25-55306BACA093}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="550" windowWidth="18090" windowHeight="16700" xr2:uid="{5A41F7F5-ACB9-4B29-8674-39A8BEA4F1FF}"/>
+    <workbookView xWindow="2220" yWindow="6700" windowWidth="26620" windowHeight="16700" xr2:uid="{5A41F7F5-ACB9-4B29-8674-39A8BEA4F1FF}"/>
   </bookViews>
   <sheets>
     <sheet name="in" sheetId="1" r:id="rId1"/>
@@ -1242,11 +1242,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1614,7 +1615,7 @@
     <col min="7" max="7" width="24.54296875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.36328125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.7265625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="23.90625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6" bestFit="1" customWidth="1"/>
@@ -1641,107 +1642,107 @@
     <col min="34" max="34" width="31.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:34" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="4" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>